<commit_message>
Incluir dominio Sí No directo en hojas de regla y actualizar ejemplo y ZIP
</commit_message>
<xml_diff>
--- a/ejemplos/reporte_prueba_excepciones.xlsx
+++ b/ejemplos/reporte_prueba_excepciones.xlsx
@@ -127,7 +127,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -146,6 +146,16 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00404040"/>
         </patternFill>
       </fill>
     </dxf>
@@ -230,22 +240,22 @@
   <commentList>
     <comment ref="G4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="H4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="I4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="J4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
   </commentList>
@@ -260,22 +270,22 @@
   <commentList>
     <comment ref="H4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="I4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="J4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="K4" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
   </commentList>
@@ -290,22 +300,22 @@
   <commentList>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>Complete primero la observación y luego escriba Sí. DT en Sí impide diligenciar los campos del operador. Los datos originales no se editan.</t>
+        <t>Seleccione Sí o No. Las observaciones se pueden diligenciar antes o después. DT en Sí oscurece toda la fila para excluirla de la revisión del operador.</t>
       </text>
     </comment>
   </commentList>
@@ -739,15 +749,6 @@
           <t>Regla incumplida: regla_prueba_01</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
-      <c r="I1" s="3" t="n"/>
-      <c r="J1" s="3" t="n"/>
     </row>
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -963,8 +964,8 @@
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:J7">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+  <conditionalFormatting sqref="A5:J7">
+    <cfRule type="expression" priority="1" dxfId="3" stopIfTrue="1">
       <formula>$G5="Sí"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -984,18 +985,12 @@
       <formula>$I5="No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation sqref="G5:G7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>OR($G5="No",AND($G5="Sí",LEN(TRIM(CLEAN(SUBSTITUTE($H5,CHAR(160)," "))))&gt;0,$I5="No",$J5=""))</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="G5:G7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Valor fuera del dominio" error="Seleccione Sí o No." promptTitle="Excepción" prompt="Seleccione Sí o No; la observación se diligencia libremente." type="list" errorStyle="stop">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>OR($G5&lt;&gt;"Sí",LEN(TRIM(CLEAN(SUBSTITUTE($H5,CHAR(160)," "))))&gt;0)</formula1>
-    </dataValidation>
-    <dataValidation sqref="I5:I7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>IF($G5="Sí",AND($I5="No",$J5=""),OR($I5="No",AND($I5="Sí",LEN(TRIM(CLEAN(SUBSTITUTE($J5,CHAR(160)," "))))&gt;0)))</formula1>
-    </dataValidation>
-    <dataValidation sqref="J5:J7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>IF($G5="Sí",$J5="",OR($I5&lt;&gt;"Sí",LEN(TRIM(CLEAN(SUBSTITUTE($J5,CHAR(160)," "))))&gt;0))</formula1>
+    <dataValidation sqref="I5:I7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Valor fuera del dominio" error="Seleccione Sí o No." promptTitle="Excepción" prompt="Seleccione Sí o No; la observación se diligencia libremente." type="list" errorStyle="stop">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1031,16 +1026,6 @@
           <t>Regla incumplida: regla_prueba_02</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
-      <c r="I1" s="3" t="n"/>
-      <c r="J1" s="3" t="n"/>
-      <c r="K1" s="3" t="n"/>
     </row>
     <row r="2" ht="54" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1223,8 +1208,8 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:K3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J5:K6">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+  <conditionalFormatting sqref="A5:K6">
+    <cfRule type="expression" priority="1" dxfId="3" stopIfTrue="1">
       <formula>$H5="Sí"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1244,18 +1229,12 @@
       <formula>$J5="No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation sqref="H5:H6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>OR($H5="No",AND($H5="Sí",LEN(TRIM(CLEAN(SUBSTITUTE($I5,CHAR(160)," "))))&gt;0,$J5="No",$K5=""))</formula1>
+  <dataValidations count="2">
+    <dataValidation sqref="H5:H6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Valor fuera del dominio" error="Seleccione Sí o No." promptTitle="Excepción" prompt="Seleccione Sí o No; la observación se diligencia libremente." type="list" errorStyle="stop">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="I5:I6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>OR($H5&lt;&gt;"Sí",LEN(TRIM(CLEAN(SUBSTITUTE($I5,CHAR(160)," "))))&gt;0)</formula1>
-    </dataValidation>
-    <dataValidation sqref="J5:J6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>IF($H5="Sí",AND($J5="No",$K5=""),OR($J5="No",AND($J5="Sí",LEN(TRIM(CLEAN(SUBSTITUTE($K5,CHAR(160)," "))))&gt;0)))</formula1>
-    </dataValidation>
-    <dataValidation sqref="K5:K6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Excepción no válida" error="Diligencie la observación antes de marcar Sí. Si DT es Sí, el operador no puede registrar excepción ni observación." promptTitle="Revisión de excepción" prompt="Escriba Sí o No. Complete primero la observación. DT en Sí bloquea los campos del operador." type="custom" errorStyle="stop">
-      <formula1>IF($H5="Sí",$K5="",OR($J5&lt;&gt;"Sí",LEN(TRIM(CLEAN(SUBSTITUTE($K5,CHAR(160)," "))))&gt;0))</formula1>
+    <dataValidation sqref="J5:J6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="Valor fuera del dominio" error="Seleccione Sí o No." promptTitle="Excepción" prompt="Seleccione Sí o No; la observación se diligencia libremente." type="list" errorStyle="stop">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1755,8 +1734,8 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <autoFilter ref="A1:R6"/>
-  <conditionalFormatting sqref="K2:L6">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+  <conditionalFormatting sqref="A2:R6">
+    <cfRule type="expression" priority="1" dxfId="3" stopIfTrue="1">
       <formula>$I2="Sí"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>